<commit_message>
Update full repository content for Nature submission: README, Reproducible_Workflow, data tables, scripts and documentation
</commit_message>
<xml_diff>
--- a/data/PMS/PMS_composition_and_overlap.xlsx
+++ b/data/PMS/PMS_composition_and_overlap.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10719"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10726"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/linweili/Important_files/课题进展/Nature_submission_rechecked_precise_red/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/linweili/Important_files/课题进展/Nature_submission_verified_red/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1B33B95-9EA9-4549-94BD-25A833CF7635}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7808BC7-810A-6F4B-8507-CEF361638DF8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="640" windowWidth="30240" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="255" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="262" uniqueCount="86">
   <si>
     <t>Marker ID</t>
   </si>
@@ -272,6 +272,12 @@
   </si>
   <si>
     <t>Extended Data Table 1 | Composition of independently curated marker sets after single-protein-tree screening</t>
+  </si>
+  <si>
+    <t>COG0199</t>
+  </si>
+  <si>
+    <t>Ribosomal protein S14</t>
   </si>
 </sst>
 </file>
@@ -602,7 +608,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H36"/>
+  <dimension ref="A1:H37"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -1180,301 +1186,325 @@
       </c>
       <c r="H24" s="19"/>
     </row>
-    <row r="25" spans="1:8" ht="34" x14ac:dyDescent="0.2">
-      <c r="A25" s="2" t="s">
+    <row r="25" spans="1:8" ht="17" x14ac:dyDescent="0.2">
+      <c r="A25" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="B25" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="C25" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="D25" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="E25" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="F25" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="G25" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="H25" s="19"/>
+    </row>
+    <row r="26" spans="1:8" ht="34" x14ac:dyDescent="0.2">
+      <c r="A26" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="B25" s="3" t="s">
+      <c r="B26" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="C25" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="D25" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="E25" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="F25" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="G25" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="H25" s="19"/>
-    </row>
-    <row r="26" spans="1:8" ht="17" x14ac:dyDescent="0.2">
-      <c r="A26" s="4" t="s">
+      <c r="C26" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="D26" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="E26" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="F26" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="G26" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="H26" s="19"/>
+    </row>
+    <row r="27" spans="1:8" ht="17" x14ac:dyDescent="0.2">
+      <c r="A27" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="B26" s="5" t="s">
+      <c r="B27" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="C26" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="D26" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="E26" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="F26" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="G26" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="H26" s="19"/>
-    </row>
-    <row r="27" spans="1:8" ht="17" x14ac:dyDescent="0.2">
-      <c r="A27" s="6" t="s">
+      <c r="C27" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="D27" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="E27" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="F27" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="G27" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="H27" s="19"/>
+    </row>
+    <row r="28" spans="1:8" ht="17" x14ac:dyDescent="0.2">
+      <c r="A28" s="6" t="s">
         <v>60</v>
       </c>
-      <c r="B27" s="7" t="s">
+      <c r="B28" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="C27" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="D27" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="E27" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="F27" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="G27" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="H27" s="18"/>
-    </row>
-    <row r="28" spans="1:8" ht="34" x14ac:dyDescent="0.2">
-      <c r="A28" s="9" t="s">
+      <c r="C28" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="D28" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="E28" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="F28" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="G28" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="H28" s="18"/>
+    </row>
+    <row r="29" spans="1:8" ht="34" x14ac:dyDescent="0.2">
+      <c r="A29" s="9" t="s">
         <v>62</v>
       </c>
-      <c r="B28" s="8" t="s">
+      <c r="B29" s="8" t="s">
         <v>63</v>
       </c>
-      <c r="C28" s="8" t="s">
-        <v>10</v>
-      </c>
-      <c r="D28" s="8" t="s">
-        <v>10</v>
-      </c>
-      <c r="E28" s="8" t="s">
-        <v>10</v>
-      </c>
-      <c r="F28" s="8" t="s">
-        <v>10</v>
-      </c>
-      <c r="G28" s="8" t="s">
-        <v>10</v>
-      </c>
-      <c r="H28" s="8" t="s">
+      <c r="C29" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="D29" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="E29" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="F29" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="G29" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="H29" s="8" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="29" spans="1:8" ht="17" x14ac:dyDescent="0.2">
-      <c r="A29" s="6" t="s">
+    <row r="30" spans="1:8" ht="17" x14ac:dyDescent="0.2">
+      <c r="A30" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="B29" s="7" t="s">
+      <c r="B30" s="7" t="s">
         <v>66</v>
       </c>
-      <c r="C29" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="D29" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="E29" s="7" t="s">
+      <c r="C30" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="D30" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="E30" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="F29" s="7" t="s">
+      <c r="F30" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="G29" s="7" t="s">
+      <c r="G30" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="H29" s="7" t="s">
+      <c r="H30" s="7" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="30" spans="1:8" ht="17" x14ac:dyDescent="0.2">
-      <c r="A30" s="4" t="s">
+    <row r="31" spans="1:8" ht="17" x14ac:dyDescent="0.2">
+      <c r="A31" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="B30" s="5" t="s">
+      <c r="B31" s="5" t="s">
         <v>69</v>
       </c>
-      <c r="C30" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="D30" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="E30" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="F30" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="G30" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="H30" s="17" t="s">
+      <c r="C31" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="D31" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="E31" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="F31" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="G31" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="H31" s="17" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="31" spans="1:8" ht="17" x14ac:dyDescent="0.2">
-      <c r="A31" s="2" t="s">
+    <row r="32" spans="1:8" ht="17" x14ac:dyDescent="0.2">
+      <c r="A32" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="B31" s="3" t="s">
+      <c r="B32" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="C31" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="D31" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="E31" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="F31" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="G31" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="H31" s="19"/>
-    </row>
-    <row r="32" spans="1:8" ht="17" x14ac:dyDescent="0.2">
-      <c r="A32" s="4" t="s">
+      <c r="C32" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="D32" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="E32" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="F32" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="G32" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="H32" s="19"/>
+    </row>
+    <row r="33" spans="1:8" ht="17" x14ac:dyDescent="0.2">
+      <c r="A33" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="B32" s="5" t="s">
+      <c r="B33" s="5" t="s">
         <v>73</v>
       </c>
-      <c r="C32" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="D32" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="E32" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="F32" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="G32" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="H32" s="19"/>
-    </row>
-    <row r="33" spans="1:8" ht="17" x14ac:dyDescent="0.2">
-      <c r="A33" s="2" t="s">
+      <c r="C33" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="D33" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="E33" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="F33" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="G33" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="H33" s="19"/>
+    </row>
+    <row r="34" spans="1:8" ht="17" x14ac:dyDescent="0.2">
+      <c r="A34" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="B33" s="3" t="s">
+      <c r="B34" s="3" t="s">
         <v>75</v>
       </c>
-      <c r="C33" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="D33" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="E33" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="F33" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="G33" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="H33" s="19"/>
-    </row>
-    <row r="34" spans="1:8" ht="17" x14ac:dyDescent="0.2">
-      <c r="A34" s="9" t="s">
+      <c r="C34" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="D34" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="E34" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="F34" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="G34" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="H34" s="19"/>
+    </row>
+    <row r="35" spans="1:8" ht="17" x14ac:dyDescent="0.2">
+      <c r="A35" s="9" t="s">
         <v>76</v>
       </c>
-      <c r="B34" s="8" t="s">
+      <c r="B35" s="8" t="s">
         <v>77</v>
       </c>
-      <c r="C34" s="8" t="s">
-        <v>10</v>
-      </c>
-      <c r="D34" s="8" t="s">
+      <c r="C35" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="D35" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="E34" s="8" t="s">
-        <v>10</v>
-      </c>
-      <c r="F34" s="8" t="s">
-        <v>10</v>
-      </c>
-      <c r="G34" s="8" t="s">
+      <c r="E35" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="F35" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="G35" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="H34" s="18"/>
-    </row>
-    <row r="35" spans="1:8" ht="34" x14ac:dyDescent="0.2">
-      <c r="A35" s="6" t="s">
+      <c r="H35" s="18"/>
+    </row>
+    <row r="36" spans="1:8" ht="34" x14ac:dyDescent="0.2">
+      <c r="A36" s="6" t="s">
         <v>78</v>
       </c>
-      <c r="B35" s="7" t="s">
+      <c r="B36" s="7" t="s">
         <v>79</v>
       </c>
-      <c r="C35" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="D35" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="E35" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="F35" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="G35" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="H35" s="7" t="s">
+      <c r="C36" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="D36" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="E36" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="F36" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="G36" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="H36" s="7" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="36" spans="1:8" ht="17" x14ac:dyDescent="0.2">
-      <c r="A36" s="10" t="s">
+    <row r="37" spans="1:8" ht="17" x14ac:dyDescent="0.2">
+      <c r="A37" s="10" t="s">
         <v>81</v>
       </c>
-      <c r="B36" s="11" t="s">
+      <c r="B37" s="11" t="s">
         <v>82</v>
       </c>
-      <c r="C36" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="D36" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="E36" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="F36" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="G36" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="H36" s="11" t="s">
+      <c r="C37" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="D37" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="E37" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="F37" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="G37" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="H37" s="11" t="s">
         <v>11</v>
       </c>
     </row>
@@ -1482,8 +1512,8 @@
   <mergeCells count="4">
     <mergeCell ref="H3:H7"/>
     <mergeCell ref="H8:H9"/>
-    <mergeCell ref="H10:H27"/>
-    <mergeCell ref="H30:H34"/>
+    <mergeCell ref="H10:H28"/>
+    <mergeCell ref="H31:H35"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>